<commit_message>
Apply triple-verification corrections to P/R workbook
Cross-checked all 5 leagues against 3+ independent official/authoritative
sources each. Corrections: France Championnat National relegation 2->3;
France National 2 relegation ~10->~8 (transition-adjusted); Spain Segunda
Federacion extra relegations made exact (2; 27 total); Italy Eccellenza
promotion tightened to ~28+7 (~35). Added verification footnote.

https://claude.ai/code/session_01NJpYPJQipfRFKUSBMkdcMH
</commit_message>
<xml_diff>
--- a/football_promotion_relegation_top5.xlsx
+++ b/football_promotion_relegation_top5.xlsx
@@ -557,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1118,12 +1118,12 @@
       </c>
       <c r="I11" s="11" t="inlineStr">
         <is>
-          <t>~2</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J11" s="11" t="inlineStr">
         <is>
-          <t>~30%</t>
+          <t>30.0%</t>
         </is>
       </c>
       <c r="K11" s="12" t="inlineStr">
@@ -1708,12 +1708,12 @@
       </c>
       <c r="F22" s="19" t="inlineStr">
         <is>
-          <t>~8</t>
+          <t>~7</t>
         </is>
       </c>
       <c r="G22" s="19" t="inlineStr">
         <is>
-          <t>~7.6%</t>
+          <t>~7.4%</t>
         </is>
       </c>
       <c r="H22" s="19" t="inlineStr">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="H25" s="23" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I25" s="23" t="inlineStr">
@@ -1893,7 +1893,7 @@
       </c>
       <c r="J25" s="23" t="inlineStr">
         <is>
-          <t>~11.1%</t>
+          <t>16.7%</t>
         </is>
       </c>
       <c r="K25" s="24" t="inlineStr">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="H26" s="23" t="inlineStr">
         <is>
-          <t>~10</t>
+          <t>~8 (variable)</t>
         </is>
       </c>
       <c r="I26" s="23" t="inlineStr">
@@ -1948,7 +1948,7 @@
       </c>
       <c r="J26" s="23" t="inlineStr">
         <is>
-          <t>~20.8%</t>
+          <t>~16.7%</t>
         </is>
       </c>
       <c r="K26" s="24" t="inlineStr">
@@ -2040,10 +2040,18 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="25" t="inlineStr">
+        <is>
+          <t>Note: All figures triple-checked (3+ independent sources per number). France is mid-transition: Championnat National relegated 3 in 2024-25 (runs at 17 clubs in 2025-26) and National 2 relegations were reduced by an FFF transition decision, so its count is variable (~8).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A30:K30"/>
     <mergeCell ref="A29:K29"/>
+    <mergeCell ref="A33:K33"/>
     <mergeCell ref="A32:K32"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A31:K31"/>

</xml_diff>